<commit_message>
Add Conroe power recliners to accent chair import
Include Cobblestone and Gray Conroe dual-power recliners with the same
8 Volusion columns, plus main/thumb/alt images under SS-CONROE-PWR-RECL
and SS-CONROE-GRAY-PWR-RECL.

Co-authored-by: emcc10 <emcc10@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/imports/steve-silver-volusion/steve_silver_accent_chairs_import.xlsx
+++ b/docs/imports/steve-silver-volusion/steve_silver_accent_chairs_import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -578,6 +578,90 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SS-CONROE-PWR-RECL</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Conroe Power Recliner</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>The Conroe Dual-Power Recliner in Cobblestone blends modern style with personalized comfort in a streamlined silhouette. Upholstered in a light tan Cobblestone fabric, it offers a warm, versatile look that fits easily into a variety of spaces. Discreet inner-arm controls allow you to independently adjust the power headrest and footrest for a fully customized lounging experience. Built with a 100% polyester cover, a durable furniture-grade plywood frame, and supportive sinuous wire springs, this recliner is designed for lasting comfort and everyday use.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>* Crafted of solid Asian hardwoods, engineered woods, foam and 100% polyester cover
+* Dual-power reclining allows you to customize your comfort with independent headrest and footrest controls, plus a convenient home button to reset the seat, located conveniently in-between seats
+* Sinuous Spring construction ensures even weight distribution, preventing the formation of sagging spots for consistent support for all seats.
+* 100% Kiln Dried Furniture-Grade Plywood frame
+* Fiber filled back provides contoured support, enhanced relaxation and resilience in an allergy-friendly fill
+* 2.0 Density Foam (in seat cushions) - Inner Bagged &amp; Baffled Fiber Fill to retain shape in seat backs
+* Durable 100% polyester cover resists wear, stains, and wrinkles while maintaining a soft, comfortable feel for everyday use.
+* 360 lb. weight capacity ensures durability and reliable support.
+* Available in Cobblestone or Gray for the Cobblestone Sectional or Gray Sectional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SS-CONROE-GRAY-PWR-RECL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Conroe Dual-Power Recliner, Gray</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>The Conroe Dual-Power Recliner in Gray blends modern style with personalized comfort in a streamlined silhouette. Upholstered in a light gray fabric, it offers a warm, versatile look that fits easily into a variety of spaces. Discreet inner-arm controls allow you to independently adjust the power headrest and footrest for a fully customized lounging experience. Built with a 100% polyester cover, a durable furniture-grade plywood frame, and supportive sinuous wire springs, this recliner is designed for lasting comfort and everyday use.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>* Crafted of solid Asian hardwoods, engineered woods, foam and 100% polyester cover
+* Dual-power reclining allows you to customize your comfort with independent headrest and footrest controls, plus a convenient home button to reset the seat, located conveniently in-between seats
+* Sinuous Spring construction ensures even weight distribution, preventing the formation of sagging spots for consistent support for all seats.
+* 100% Kiln Dried Furniture-Grade Plywood frame
+* Fiber filled back provides contoured support, enhanced relaxation and resilience in an allergy-friendly fill
+* 2.0 Density Foam (in seat cushions) - Inner Bagged &amp; Baffled Fiber Fill to retain shape in seat backs
+* Durable 100% polyester cover resists wear, stains, and wrinkles while maintaining a soft, comfortable feel for everyday use.
+* 360 lb. weight capacity ensures durability and reliable support.
+* Available in Cobblestone or Gray for the Cobblestone Sectional or Gray Sectional.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>